<commit_message>
data: 2026-09-14 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I77"/>
+  <dimension ref="A1:I78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2834,6 +2834,37 @@
         <v>96.73</v>
       </c>
     </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B78" s="3" t="n">
+        <v>9051</v>
+      </c>
+      <c r="C78" s="3" t="n">
+        <v>10384374.32</v>
+      </c>
+      <c r="D78" s="3" t="n">
+        <v>9138884.560000001</v>
+      </c>
+      <c r="E78" s="3" t="n">
+        <v>1245489.75</v>
+      </c>
+      <c r="F78" s="4" t="n">
+        <v>3.8878</v>
+      </c>
+      <c r="G78" s="4" t="n">
+        <v>1147.32</v>
+      </c>
+      <c r="H78" s="5" t="n">
+        <v>83.08</v>
+      </c>
+      <c r="I78" s="5" t="n">
+        <v>96.73</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-09-15 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I78"/>
+  <dimension ref="A1:I79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2865,6 +2865,37 @@
         <v>96.73</v>
       </c>
     </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B79" s="3" t="n">
+        <v>9045</v>
+      </c>
+      <c r="C79" s="3" t="n">
+        <v>10390035.12</v>
+      </c>
+      <c r="D79" s="3" t="n">
+        <v>9152214.529999999</v>
+      </c>
+      <c r="E79" s="3" t="n">
+        <v>1237820.59</v>
+      </c>
+      <c r="F79" s="4" t="n">
+        <v>3.8878</v>
+      </c>
+      <c r="G79" s="4" t="n">
+        <v>1148.7</v>
+      </c>
+      <c r="H79" s="5" t="n">
+        <v>83.04000000000001</v>
+      </c>
+      <c r="I79" s="5" t="n">
+        <v>96.70999999999999</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-09-16 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I79"/>
+  <dimension ref="A1:I80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2896,6 +2896,37 @@
         <v>96.70999999999999</v>
       </c>
     </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B80" s="3" t="n">
+        <v>9042</v>
+      </c>
+      <c r="C80" s="3" t="n">
+        <v>10384839.88</v>
+      </c>
+      <c r="D80" s="3" t="n">
+        <v>9153194.02</v>
+      </c>
+      <c r="E80" s="3" t="n">
+        <v>1231645.86</v>
+      </c>
+      <c r="F80" s="4" t="n">
+        <v>3.892</v>
+      </c>
+      <c r="G80" s="4" t="n">
+        <v>1148.51</v>
+      </c>
+      <c r="H80" s="5" t="n">
+        <v>83.06999999999999</v>
+      </c>
+      <c r="I80" s="5" t="n">
+        <v>96.75</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-09-17 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I80"/>
+  <dimension ref="A1:I81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2927,6 +2927,37 @@
         <v>96.75</v>
       </c>
     </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B81" s="3" t="n">
+        <v>9040</v>
+      </c>
+      <c r="C81" s="3" t="n">
+        <v>10382904.89</v>
+      </c>
+      <c r="D81" s="3" t="n">
+        <v>9148989.84</v>
+      </c>
+      <c r="E81" s="3" t="n">
+        <v>1233915.05</v>
+      </c>
+      <c r="F81" s="4" t="n">
+        <v>3.9046</v>
+      </c>
+      <c r="G81" s="4" t="n">
+        <v>1148.55</v>
+      </c>
+      <c r="H81" s="5" t="n">
+        <v>83.09</v>
+      </c>
+      <c r="I81" s="5" t="n">
+        <v>96.73999999999999</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-09-18 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I81"/>
+  <dimension ref="A1:I82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2958,6 +2958,37 @@
         <v>96.73999999999999</v>
       </c>
     </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B82" s="3" t="n">
+        <v>9040</v>
+      </c>
+      <c r="C82" s="3" t="n">
+        <v>10338566.37</v>
+      </c>
+      <c r="D82" s="3" t="n">
+        <v>9098763.279999999</v>
+      </c>
+      <c r="E82" s="3" t="n">
+        <v>1239803.1</v>
+      </c>
+      <c r="F82" s="4" t="n">
+        <v>3.9007</v>
+      </c>
+      <c r="G82" s="4" t="n">
+        <v>1143.65</v>
+      </c>
+      <c r="H82" s="5" t="n">
+        <v>82.95999999999999</v>
+      </c>
+      <c r="I82" s="5" t="n">
+        <v>96.72</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-09-19 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I82"/>
+  <dimension ref="A1:I83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2989,6 +2989,37 @@
         <v>96.72</v>
       </c>
     </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="B83" s="3" t="n">
+        <v>9064</v>
+      </c>
+      <c r="C83" s="3" t="n">
+        <v>10343122.35</v>
+      </c>
+      <c r="D83" s="3" t="n">
+        <v>9094885.07</v>
+      </c>
+      <c r="E83" s="3" t="n">
+        <v>1248237.28</v>
+      </c>
+      <c r="F83" s="4" t="n">
+        <v>3.9257</v>
+      </c>
+      <c r="G83" s="4" t="n">
+        <v>1141.12</v>
+      </c>
+      <c r="H83" s="5" t="n">
+        <v>82.92</v>
+      </c>
+      <c r="I83" s="5" t="n">
+        <v>96.69</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-09-20 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I83"/>
+  <dimension ref="A1:I84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3020,6 +3020,37 @@
         <v>96.69</v>
       </c>
     </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B84" s="3" t="n">
+        <v>9064</v>
+      </c>
+      <c r="C84" s="3" t="n">
+        <v>10343497.33</v>
+      </c>
+      <c r="D84" s="3" t="n">
+        <v>9094972.029999999</v>
+      </c>
+      <c r="E84" s="3" t="n">
+        <v>1248525.3</v>
+      </c>
+      <c r="F84" s="4" t="n">
+        <v>3.9385</v>
+      </c>
+      <c r="G84" s="4" t="n">
+        <v>1141.16</v>
+      </c>
+      <c r="H84" s="5" t="n">
+        <v>82.92</v>
+      </c>
+      <c r="I84" s="5" t="n">
+        <v>96.68000000000001</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-09-21 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I84"/>
+  <dimension ref="A1:I85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3051,6 +3051,37 @@
         <v>96.68000000000001</v>
       </c>
     </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B85" s="3" t="n">
+        <v>9067</v>
+      </c>
+      <c r="C85" s="3" t="n">
+        <v>10345035.23</v>
+      </c>
+      <c r="D85" s="3" t="n">
+        <v>9093863.369999999</v>
+      </c>
+      <c r="E85" s="3" t="n">
+        <v>1251171.86</v>
+      </c>
+      <c r="F85" s="4" t="n">
+        <v>3.9311</v>
+      </c>
+      <c r="G85" s="4" t="n">
+        <v>1140.95</v>
+      </c>
+      <c r="H85" s="5" t="n">
+        <v>82.90000000000001</v>
+      </c>
+      <c r="I85" s="5" t="n">
+        <v>96.73</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-09-22 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I85"/>
+  <dimension ref="A1:I86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3082,6 +3082,37 @@
         <v>96.73</v>
       </c>
     </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B86" s="3" t="n">
+        <v>9088</v>
+      </c>
+      <c r="C86" s="3" t="n">
+        <v>10363418.51</v>
+      </c>
+      <c r="D86" s="3" t="n">
+        <v>9098214.76</v>
+      </c>
+      <c r="E86" s="3" t="n">
+        <v>1265203.76</v>
+      </c>
+      <c r="F86" s="4" t="n">
+        <v>3.9157</v>
+      </c>
+      <c r="G86" s="4" t="n">
+        <v>1140.34</v>
+      </c>
+      <c r="H86" s="5" t="n">
+        <v>82.75</v>
+      </c>
+      <c r="I86" s="5" t="n">
+        <v>96.68000000000001</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-09-23 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I86"/>
+  <dimension ref="A1:I87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3113,6 +3113,37 @@
         <v>96.68000000000001</v>
       </c>
     </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B87" s="3" t="n">
+        <v>9097</v>
+      </c>
+      <c r="C87" s="3" t="n">
+        <v>10390217.36</v>
+      </c>
+      <c r="D87" s="3" t="n">
+        <v>9097882.42</v>
+      </c>
+      <c r="E87" s="3" t="n">
+        <v>1292334.94</v>
+      </c>
+      <c r="F87" s="4" t="n">
+        <v>3.9031</v>
+      </c>
+      <c r="G87" s="4" t="n">
+        <v>1142.16</v>
+      </c>
+      <c r="H87" s="5" t="n">
+        <v>82.54000000000001</v>
+      </c>
+      <c r="I87" s="5" t="n">
+        <v>96.65000000000001</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-09-24 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I87"/>
+  <dimension ref="A1:I88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3144,6 +3144,37 @@
         <v>96.65000000000001</v>
       </c>
     </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B88" s="3" t="n">
+        <v>9082</v>
+      </c>
+      <c r="C88" s="3" t="n">
+        <v>10376448.96</v>
+      </c>
+      <c r="D88" s="3" t="n">
+        <v>9097319</v>
+      </c>
+      <c r="E88" s="3" t="n">
+        <v>1279129.97</v>
+      </c>
+      <c r="F88" s="4" t="n">
+        <v>3.8939</v>
+      </c>
+      <c r="G88" s="4" t="n">
+        <v>1142.53</v>
+      </c>
+      <c r="H88" s="5" t="n">
+        <v>82.65000000000001</v>
+      </c>
+      <c r="I88" s="5" t="n">
+        <v>96.66</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-09-25 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I88"/>
+  <dimension ref="A1:I89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3175,6 +3175,37 @@
         <v>96.66</v>
       </c>
     </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B89" s="3" t="n">
+        <v>9088</v>
+      </c>
+      <c r="C89" s="3" t="n">
+        <v>10314113.91</v>
+      </c>
+      <c r="D89" s="3" t="n">
+        <v>9094051.49</v>
+      </c>
+      <c r="E89" s="3" t="n">
+        <v>1220062.42</v>
+      </c>
+      <c r="F89" s="4" t="n">
+        <v>3.9031</v>
+      </c>
+      <c r="G89" s="4" t="n">
+        <v>1134.92</v>
+      </c>
+      <c r="H89" s="5" t="n">
+        <v>83.14</v>
+      </c>
+      <c r="I89" s="5" t="n">
+        <v>96.63</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-09-26 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I89"/>
+  <dimension ref="A1:I90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3206,6 +3206,37 @@
         <v>96.63</v>
       </c>
     </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="B90" s="3" t="n">
+        <v>9097</v>
+      </c>
+      <c r="C90" s="3" t="n">
+        <v>10316289.98</v>
+      </c>
+      <c r="D90" s="3" t="n">
+        <v>9095003.369999999</v>
+      </c>
+      <c r="E90" s="3" t="n">
+        <v>1221286.62</v>
+      </c>
+      <c r="F90" s="4" t="n">
+        <v>3.9073</v>
+      </c>
+      <c r="G90" s="4" t="n">
+        <v>1134.03</v>
+      </c>
+      <c r="H90" s="5" t="n">
+        <v>83.12</v>
+      </c>
+      <c r="I90" s="5" t="n">
+        <v>96.62</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-09-27 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I90"/>
+  <dimension ref="A1:I91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3237,6 +3237,37 @@
         <v>96.62</v>
       </c>
     </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B91" s="3" t="n">
+        <v>9129</v>
+      </c>
+      <c r="C91" s="3" t="n">
+        <v>10306323.46</v>
+      </c>
+      <c r="D91" s="3" t="n">
+        <v>9094820.23</v>
+      </c>
+      <c r="E91" s="3" t="n">
+        <v>1211503.23</v>
+      </c>
+      <c r="F91" s="4" t="n">
+        <v>3.9353</v>
+      </c>
+      <c r="G91" s="4" t="n">
+        <v>1128.97</v>
+      </c>
+      <c r="H91" s="5" t="n">
+        <v>83.2</v>
+      </c>
+      <c r="I91" s="5" t="n">
+        <v>96.64</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-09-28 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I91"/>
+  <dimension ref="A1:I92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3268,6 +3268,37 @@
         <v>96.64</v>
       </c>
     </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B92" s="3" t="n">
+        <v>9228</v>
+      </c>
+      <c r="C92" s="3" t="n">
+        <v>10302368.26</v>
+      </c>
+      <c r="D92" s="3" t="n">
+        <v>9088328.789999999</v>
+      </c>
+      <c r="E92" s="3" t="n">
+        <v>1214039.47</v>
+      </c>
+      <c r="F92" s="4" t="n">
+        <v>3.7928</v>
+      </c>
+      <c r="G92" s="4" t="n">
+        <v>1116.42</v>
+      </c>
+      <c r="H92" s="5" t="n">
+        <v>83.18000000000001</v>
+      </c>
+      <c r="I92" s="5" t="n">
+        <v>96.63</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-09-29 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I92"/>
+  <dimension ref="A1:I93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3299,6 +3299,37 @@
         <v>96.63</v>
       </c>
     </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B93" s="3" t="n">
+        <v>9229</v>
+      </c>
+      <c r="C93" s="3" t="n">
+        <v>10299845.66</v>
+      </c>
+      <c r="D93" s="3" t="n">
+        <v>9094065.890000001</v>
+      </c>
+      <c r="E93" s="3" t="n">
+        <v>1205779.77</v>
+      </c>
+      <c r="F93" s="4" t="n">
+        <v>3.7895</v>
+      </c>
+      <c r="G93" s="4" t="n">
+        <v>1116.03</v>
+      </c>
+      <c r="H93" s="5" t="n">
+        <v>83.2</v>
+      </c>
+      <c r="I93" s="5" t="n">
+        <v>96.63</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-09-30 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I93"/>
+  <dimension ref="A1:I94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3330,6 +3330,37 @@
         <v>96.63</v>
       </c>
     </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B94" s="3" t="n">
+        <v>9109</v>
+      </c>
+      <c r="C94" s="3" t="n">
+        <v>10298396.71</v>
+      </c>
+      <c r="D94" s="3" t="n">
+        <v>9093828.550000001</v>
+      </c>
+      <c r="E94" s="3" t="n">
+        <v>1204568.16</v>
+      </c>
+      <c r="F94" s="4" t="n">
+        <v>3.9073</v>
+      </c>
+      <c r="G94" s="4" t="n">
+        <v>1130.57</v>
+      </c>
+      <c r="H94" s="5" t="n">
+        <v>86.04000000000001</v>
+      </c>
+      <c r="I94" s="5" t="n">
+        <v>96.69</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-10-01 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I94"/>
+  <dimension ref="A1:I95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3361,6 +3361,37 @@
         <v>96.69</v>
       </c>
     </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="B95" s="3" t="n">
+        <v>9107</v>
+      </c>
+      <c r="C95" s="3" t="n">
+        <v>10148416.48</v>
+      </c>
+      <c r="D95" s="3" t="n">
+        <v>9093970.67</v>
+      </c>
+      <c r="E95" s="3" t="n">
+        <v>1054445.81</v>
+      </c>
+      <c r="F95" s="4" t="n">
+        <v>3.9054</v>
+      </c>
+      <c r="G95" s="4" t="n">
+        <v>1114.35</v>
+      </c>
+      <c r="H95" s="5" t="n">
+        <v>86.86</v>
+      </c>
+      <c r="I95" s="5" t="n">
+        <v>96.65000000000001</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-10-02 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I95"/>
+  <dimension ref="A1:I96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3392,6 +3392,37 @@
         <v>96.65000000000001</v>
       </c>
     </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B96" s="3" t="n">
+        <v>9114</v>
+      </c>
+      <c r="C96" s="3" t="n">
+        <v>10146967.93</v>
+      </c>
+      <c r="D96" s="3" t="n">
+        <v>9093248.720000001</v>
+      </c>
+      <c r="E96" s="3" t="n">
+        <v>1053719.21</v>
+      </c>
+      <c r="F96" s="4" t="n">
+        <v>3.9095</v>
+      </c>
+      <c r="G96" s="4" t="n">
+        <v>1113.34</v>
+      </c>
+      <c r="H96" s="5" t="n">
+        <v>86.87</v>
+      </c>
+      <c r="I96" s="5" t="n">
+        <v>96.66</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-10-03 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I96"/>
+  <dimension ref="A1:I97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3423,6 +3423,37 @@
         <v>96.66</v>
       </c>
     </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B97" s="3" t="n">
+        <v>9114</v>
+      </c>
+      <c r="C97" s="3" t="n">
+        <v>10153059.54</v>
+      </c>
+      <c r="D97" s="3" t="n">
+        <v>9095343.779999999</v>
+      </c>
+      <c r="E97" s="3" t="n">
+        <v>1057715.75</v>
+      </c>
+      <c r="F97" s="4" t="n">
+        <v>3.9073</v>
+      </c>
+      <c r="G97" s="4" t="n">
+        <v>1114.01</v>
+      </c>
+      <c r="H97" s="5" t="n">
+        <v>86.81999999999999</v>
+      </c>
+      <c r="I97" s="5" t="n">
+        <v>96.63</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-10-04 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I97"/>
+  <dimension ref="A1:I98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3454,6 +3454,37 @@
         <v>96.63</v>
       </c>
     </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B98" s="3" t="n">
+        <v>9114</v>
+      </c>
+      <c r="C98" s="3" t="n">
+        <v>10146540.35</v>
+      </c>
+      <c r="D98" s="3" t="n">
+        <v>9088360.130000001</v>
+      </c>
+      <c r="E98" s="3" t="n">
+        <v>1058180.22</v>
+      </c>
+      <c r="F98" s="4" t="n">
+        <v>3.9073</v>
+      </c>
+      <c r="G98" s="4" t="n">
+        <v>1113.29</v>
+      </c>
+      <c r="H98" s="5" t="n">
+        <v>86.81</v>
+      </c>
+      <c r="I98" s="5" t="n">
+        <v>96.63</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
data: 2026-10-05 — flow + holders + activity
</commit_message>
<xml_diff>
--- a/KUB_Holders_Daily.xlsx
+++ b/KUB_Holders_Daily.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I98"/>
+  <dimension ref="A1:I99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3485,6 +3485,37 @@
         <v>96.63</v>
       </c>
     </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="B99" s="3" t="n">
+        <v>9117</v>
+      </c>
+      <c r="C99" s="3" t="n">
+        <v>10146338.2</v>
+      </c>
+      <c r="D99" s="3" t="n">
+        <v>9088018.26</v>
+      </c>
+      <c r="E99" s="3" t="n">
+        <v>1058319.94</v>
+      </c>
+      <c r="F99" s="4" t="n">
+        <v>3.9055</v>
+      </c>
+      <c r="G99" s="4" t="n">
+        <v>1112.9</v>
+      </c>
+      <c r="H99" s="5" t="n">
+        <v>86.81</v>
+      </c>
+      <c r="I99" s="5" t="n">
+        <v>96.62</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>